<commit_message>
Update of READ.md file
</commit_message>
<xml_diff>
--- a/Lab-trails/2026-04-29-CattleSlurryRetry-picarro.xlsx
+++ b/Lab-trails/2026-04-29-CattleSlurryRetry-picarro.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\2026-04-29-cattle-slurry-retrail\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mikae\Desktop\Github - speciale\Larsen-2025-Masterthesis-DFCs\Lab-trails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6E7EE3-C9D5-455F-AED1-C279FBB9B92D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1AE0054-FEF3-482B-836C-94741575B348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="28">
   <si>
     <t>Valve code</t>
   </si>
@@ -150,16 +150,23 @@
   </si>
   <si>
     <t>endtime</t>
+  </si>
+  <si>
+    <t>Mean</t>
+  </si>
+  <si>
+    <t>stdev</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,12 +179,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -222,7 +223,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -523,7 +524,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
@@ -540,7 +541,7 @@
     <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -589,8 +590,14 @@
       <c r="P1" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -622,7 +629,7 @@
       <c r="J2" s="1">
         <v>0.95199999999999996</v>
       </c>
-      <c r="K2" s="9">
+      <c r="K2" s="1">
         <f>I2+J2</f>
         <v>1.1739999999999999</v>
       </c>
@@ -642,8 +649,16 @@
       <c r="P2" s="2">
         <v>0.59652777777777777</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="R2" s="1">
+        <f>AVERAGE(E2:E24)</f>
+        <v>2.0458499999999997</v>
+      </c>
+      <c r="S2">
+        <f>_xlfn.STDEV.P(E2:E25)</f>
+        <v>2.9156945999195511E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -675,7 +690,7 @@
       <c r="J3" s="1">
         <v>0.96299999999999997</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="1">
         <f t="shared" ref="K3:K25" si="1">I3+J3</f>
         <v>1.1759999999999999</v>
       </c>
@@ -684,7 +699,7 @@
         <v>1.1844999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -716,7 +731,7 @@
       <c r="J4" s="1">
         <v>0.96599999999999997</v>
       </c>
-      <c r="K4" s="9">
+      <c r="K4" s="1">
         <f t="shared" si="1"/>
         <v>1.177</v>
       </c>
@@ -724,8 +739,12 @@
         <f t="shared" si="2"/>
         <v>1.1840000000000002</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="N4" s="9">
+        <f>AVERAGE(L2:L25)</f>
+        <v>1.2161249999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -757,7 +776,7 @@
       <c r="J5" s="1">
         <v>0.96599999999999997</v>
       </c>
-      <c r="K5" s="9">
+      <c r="K5" s="1">
         <f t="shared" si="1"/>
         <v>1.175</v>
       </c>
@@ -765,8 +784,12 @@
         <f t="shared" si="2"/>
         <v>1.5514999999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="N5" s="9">
+        <f>_xlfn.STDEV.P(L2:L25)</f>
+        <v>0.1010966173601603</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -798,7 +821,7 @@
       <c r="J6" s="1">
         <v>0.96099999999999997</v>
       </c>
-      <c r="K6" s="9">
+      <c r="K6" s="1">
         <f t="shared" si="1"/>
         <v>1.171</v>
       </c>
@@ -807,7 +830,7 @@
         <v>1.5505</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>11</v>
       </c>
@@ -848,7 +871,7 @@
         <v>1.2065000000000001</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>6</v>
       </c>
@@ -877,7 +900,7 @@
       <c r="J8" s="1">
         <v>0.96499999999999997</v>
       </c>
-      <c r="K8" s="9">
+      <c r="K8" s="1">
         <f t="shared" si="1"/>
         <v>1.175</v>
       </c>
@@ -886,7 +909,7 @@
         <v>1.1830000000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>7</v>
       </c>
@@ -915,7 +938,7 @@
       <c r="J9" s="1">
         <v>0.96499999999999997</v>
       </c>
-      <c r="K9" s="9">
+      <c r="K9" s="1">
         <f t="shared" si="1"/>
         <v>1.177</v>
       </c>
@@ -924,7 +947,7 @@
         <v>1.1844999999999999</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>8</v>
       </c>
@@ -953,7 +976,7 @@
       <c r="J10" s="1">
         <v>0.96199999999999997</v>
       </c>
-      <c r="K10" s="9">
+      <c r="K10" s="1">
         <f t="shared" si="1"/>
         <v>1.177</v>
       </c>
@@ -962,7 +985,7 @@
         <v>1.1844999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>9</v>
       </c>
@@ -991,7 +1014,7 @@
       <c r="J11" s="1">
         <v>0.96299999999999997</v>
       </c>
-      <c r="K11" s="9">
+      <c r="K11" s="1">
         <f t="shared" si="1"/>
         <v>1.1759999999999999</v>
       </c>
@@ -1000,7 +1023,7 @@
         <v>1.1844999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>10</v>
       </c>
@@ -1029,7 +1052,7 @@
       <c r="J12" s="1">
         <v>0.96099999999999997</v>
       </c>
-      <c r="K12" s="9">
+      <c r="K12" s="1">
         <f t="shared" si="1"/>
         <v>1.177</v>
       </c>
@@ -1038,7 +1061,7 @@
         <v>1.1844999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1079,7 +1102,7 @@
         <v>1.1915</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>16</v>
       </c>
@@ -1111,7 +1134,7 @@
       <c r="J14" s="1">
         <v>0.96199999999999997</v>
       </c>
-      <c r="K14" s="9">
+      <c r="K14" s="1">
         <f t="shared" si="1"/>
         <v>1.1739999999999999</v>
       </c>
@@ -1120,7 +1143,7 @@
         <v>1.1839999999999999</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>16</v>
       </c>
@@ -1152,7 +1175,7 @@
       <c r="J15" s="1">
         <v>0.97599999999999998</v>
       </c>
-      <c r="K15" s="9">
+      <c r="K15" s="1">
         <f t="shared" si="1"/>
         <v>1.1739999999999999</v>
       </c>
@@ -1161,7 +1184,7 @@
         <v>1.1835</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>16</v>
       </c>
@@ -1193,7 +1216,7 @@
       <c r="J16" s="1">
         <v>1.0309999999999999</v>
       </c>
-      <c r="K16" s="9">
+      <c r="K16" s="1">
         <f t="shared" si="1"/>
         <v>1.1709999999999998</v>
       </c>
@@ -1234,7 +1257,7 @@
       <c r="J17" s="1">
         <v>0.96699999999999997</v>
       </c>
-      <c r="K17" s="9">
+      <c r="K17" s="1">
         <f t="shared" si="1"/>
         <v>1.175</v>
       </c>
@@ -1275,7 +1298,7 @@
       <c r="J18" s="1">
         <v>0.96099999999999997</v>
       </c>
-      <c r="K18" s="9">
+      <c r="K18" s="1">
         <f t="shared" si="1"/>
         <v>1.175</v>
       </c>
@@ -1357,7 +1380,7 @@
       <c r="J20" s="1">
         <v>0.97199999999999998</v>
       </c>
-      <c r="K20" s="9">
+      <c r="K20" s="1">
         <f t="shared" si="1"/>
         <v>1.1739999999999999</v>
       </c>
@@ -1398,7 +1421,7 @@
       <c r="J21" s="1">
         <v>0.96399999999999997</v>
       </c>
-      <c r="K21" s="9">
+      <c r="K21" s="1">
         <f t="shared" si="1"/>
         <v>1.1739999999999999</v>
       </c>
@@ -1439,7 +1462,7 @@
       <c r="J22" s="1">
         <v>0.97899999999999998</v>
       </c>
-      <c r="K22" s="9">
+      <c r="K22" s="1">
         <f t="shared" si="1"/>
         <v>1.1759999999999999</v>
       </c>
@@ -1480,7 +1503,7 @@
       <c r="J23" s="1">
         <v>0.96099999999999997</v>
       </c>
-      <c r="K23" s="9">
+      <c r="K23" s="1">
         <f t="shared" si="1"/>
         <v>1.1759999999999999</v>
       </c>
@@ -1521,7 +1544,7 @@
       <c r="J24" s="1">
         <v>0.96699999999999997</v>
       </c>
-      <c r="K24" s="9">
+      <c r="K24" s="1">
         <f t="shared" si="1"/>
         <v>1.175</v>
       </c>

</xml_diff>